<commit_message>
Enhance molecular optimization framework by introducing a neural network model for predicting energetic material properties. Implement training and prediction functions using Coulomb matrix eigenvalue descriptors, including multi-output capabilities. Update retraining scripts to support the new neural network approach and ensure compatibility with existing models. Refactor GUI components to display prediction results effectively and improve user interaction. Adjust sample input files for consistency with new prediction methods.
</commit_message>
<xml_diff>
--- a/prediction results.xlsx
+++ b/prediction results.xlsx
@@ -1,31 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PycharmProjects\EnergeticGraph\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cursor Projects\EnergeticGraph\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97CE8409-34B7-4601-A6A1-0032C4ABDE2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07049A9-07FD-45BF-93C6-6ABD6146BDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="31785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6660" yWindow="6100" windowWidth="28800" windowHeight="15370" activeTab="4" xr2:uid="{89EC946F-DC53-429F-91F6-32650855A236}"/>
   </bookViews>
   <sheets>
-    <sheet name="KernelRidge" sheetId="1" r:id="rId1"/>
+    <sheet name="Kernel Ridge" sheetId="1" r:id="rId1"/>
+    <sheet name="SVR" sheetId="2" r:id="rId2"/>
+    <sheet name="Random Forest" sheetId="3" r:id="rId3"/>
+    <sheet name="XGBoost" sheetId="4" r:id="rId4"/>
+    <sheet name="XGBoost (Coulomb)" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="12">
   <si>
     <t>property</t>
   </si>
@@ -71,16 +86,15 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -100,19 +114,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Excel Built-in Normal" xfId="1" xr:uid="{7517A7B9-DA41-4492-AC62-95B9CBCEB1EB}"/>
+    <cellStyle name="Excel Built-in Percent" xfId="2" xr:uid="{744D70DF-7DDE-473D-8014-99E02BAEC3D9}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -138,39 +151,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -203,9 +216,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -238,6 +268,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -299,13 +346,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -314,6 +354,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -378,30 +425,50 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{162FD3F5-A2F3-4737-B403-30054D213DAE}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -421,124 +488,756 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2">
         <v>0.88800000000000001</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2">
         <v>0.77569999999999995</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2">
         <v>6.5799999999999997E-2</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2">
         <v>4.0099999999999997E-2</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2">
         <v>5.4399999999999997E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <v>0.98129999999999995</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3">
         <v>0.95230000000000004</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3">
         <v>292.40589999999997</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3">
         <v>231.30420000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>0.75539999999999996</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4">
         <v>0.56979999999999997</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4">
         <v>76.335499999999996</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>0.1113</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4">
         <v>50.082799999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>0.97789999999999999</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5">
         <v>0.94199999999999995</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5">
         <v>2.0305</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5">
         <v>0.1008</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5">
         <v>1.5709</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6">
         <v>0.92320000000000002</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6">
         <v>0.86019999999999996</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6">
         <v>627.75739999999996</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6">
         <v>0.14710000000000001</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6">
         <v>457.5496</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>0.94430000000000003</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>0.79400000000000004</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7">
         <v>173.37459999999999</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7">
         <v>0.76739999999999997</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7">
         <v>114.2212</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{719D0C69-70FA-48C5-B803-41A9A261E93C}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0.87639999999999996</v>
+      </c>
+      <c r="C2">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="D2">
+        <v>5.9200000000000003E-2</v>
+      </c>
+      <c r="E2">
+        <v>3.6200000000000003E-2</v>
+      </c>
+      <c r="F2">
+        <v>4.7699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>0.93920000000000003</v>
+      </c>
+      <c r="C3">
+        <v>0.91549999999999998</v>
+      </c>
+      <c r="D3">
+        <v>388.87860000000001</v>
+      </c>
+      <c r="E3">
+        <v>5.7799999999999997E-2</v>
+      </c>
+      <c r="F3">
+        <v>291.76839999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>0.72340000000000004</v>
+      </c>
+      <c r="C4">
+        <v>0.28820000000000001</v>
+      </c>
+      <c r="D4">
+        <v>98.194900000000004</v>
+      </c>
+      <c r="E4">
+        <v>0.14319999999999999</v>
+      </c>
+      <c r="F4">
+        <v>54.759500000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>0.97699999999999998</v>
+      </c>
+      <c r="C5">
+        <v>0.93420000000000003</v>
+      </c>
+      <c r="D5">
+        <v>2.1627000000000001</v>
+      </c>
+      <c r="E5">
+        <v>0.10730000000000001</v>
+      </c>
+      <c r="F5">
+        <v>1.6527000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0.73180000000000001</v>
+      </c>
+      <c r="C6">
+        <v>0.66879999999999995</v>
+      </c>
+      <c r="D6">
+        <v>966.25300000000004</v>
+      </c>
+      <c r="E6">
+        <v>0.22650000000000001</v>
+      </c>
+      <c r="F6">
+        <v>691.13220000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>0.67559999999999998</v>
+      </c>
+      <c r="C7">
+        <v>0.59430000000000005</v>
+      </c>
+      <c r="D7">
+        <v>243.2944</v>
+      </c>
+      <c r="E7">
+        <v>1.0768</v>
+      </c>
+      <c r="F7">
+        <v>171.20609999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9925CAE-27CB-45B8-BB86-BFB93AAA30D8}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0.94259999999999999</v>
+      </c>
+      <c r="C2">
+        <v>0.82010000000000005</v>
+      </c>
+      <c r="D2">
+        <v>5.8900000000000001E-2</v>
+      </c>
+      <c r="E2">
+        <v>3.5900000000000001E-2</v>
+      </c>
+      <c r="F2">
+        <v>4.65E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>0.99239999999999995</v>
+      </c>
+      <c r="C3">
+        <v>0.95679999999999998</v>
+      </c>
+      <c r="D3">
+        <v>278.21260000000001</v>
+      </c>
+      <c r="E3">
+        <v>4.1399999999999999E-2</v>
+      </c>
+      <c r="F3">
+        <v>217.05670000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>0.95930000000000004</v>
+      </c>
+      <c r="C4">
+        <v>0.67430000000000001</v>
+      </c>
+      <c r="D4">
+        <v>66.418499999999995</v>
+      </c>
+      <c r="E4">
+        <v>9.6799999999999997E-2</v>
+      </c>
+      <c r="F4">
+        <v>36.166800000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="C5">
+        <v>0.95250000000000001</v>
+      </c>
+      <c r="D5">
+        <v>1.8374999999999999</v>
+      </c>
+      <c r="E5">
+        <v>9.1200000000000003E-2</v>
+      </c>
+      <c r="F5">
+        <v>1.4157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0.97160000000000002</v>
+      </c>
+      <c r="C6">
+        <v>0.83950000000000002</v>
+      </c>
+      <c r="D6">
+        <v>672.69640000000004</v>
+      </c>
+      <c r="E6">
+        <v>0.15770000000000001</v>
+      </c>
+      <c r="F6">
+        <v>487.69139999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>0.97289999999999999</v>
+      </c>
+      <c r="C7">
+        <v>0.76580000000000004</v>
+      </c>
+      <c r="D7">
+        <v>184.87350000000001</v>
+      </c>
+      <c r="E7">
+        <v>0.81830000000000003</v>
+      </c>
+      <c r="F7">
+        <v>116.2313</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FED6D5C-92F2-433E-A07F-C9221DC9F56E}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0.92769999999999997</v>
+      </c>
+      <c r="C2">
+        <v>0.79569999999999996</v>
+      </c>
+      <c r="D2">
+        <v>6.4799999999999996E-2</v>
+      </c>
+      <c r="E2">
+        <v>3.9399999999999998E-2</v>
+      </c>
+      <c r="F2">
+        <v>5.1799999999999999E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="C3">
+        <v>0.95820000000000005</v>
+      </c>
+      <c r="D3">
+        <v>301.88080000000002</v>
+      </c>
+      <c r="E3">
+        <v>4.4299999999999999E-2</v>
+      </c>
+      <c r="F3">
+        <v>200.01070000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>0.87080000000000002</v>
+      </c>
+      <c r="C4">
+        <v>0.66190000000000004</v>
+      </c>
+      <c r="D4">
+        <v>61.226300000000002</v>
+      </c>
+      <c r="E4">
+        <v>8.7599999999999997E-2</v>
+      </c>
+      <c r="F4">
+        <v>39.7517</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>0.99260000000000004</v>
+      </c>
+      <c r="C5">
+        <v>0.94159999999999999</v>
+      </c>
+      <c r="D5">
+        <v>2.1560000000000001</v>
+      </c>
+      <c r="E5">
+        <v>0.1045</v>
+      </c>
+      <c r="F5">
+        <v>1.3153999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0.95420000000000005</v>
+      </c>
+      <c r="C6">
+        <v>0.85089999999999999</v>
+      </c>
+      <c r="D6">
+        <v>593.97299999999996</v>
+      </c>
+      <c r="E6">
+        <v>0.13739999999999999</v>
+      </c>
+      <c r="F6">
+        <v>478.46690000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>0.96619999999999995</v>
+      </c>
+      <c r="C7">
+        <v>0.83220000000000005</v>
+      </c>
+      <c r="D7">
+        <v>144.36969999999999</v>
+      </c>
+      <c r="E7">
+        <v>0.57740000000000002</v>
+      </c>
+      <c r="F7">
+        <v>110.27249999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689E851C-92EB-4238-AD5F-CA3B296E8810}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0.98009999999999997</v>
+      </c>
+      <c r="C2">
+        <v>0.81299999999999994</v>
+      </c>
+      <c r="D2">
+        <v>6.2E-2</v>
+      </c>
+      <c r="E2">
+        <v>3.7699999999999997E-2</v>
+      </c>
+      <c r="F2">
+        <v>4.7600000000000003E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>0.89029999999999998</v>
+      </c>
+      <c r="D3">
+        <v>489.19229999999999</v>
+      </c>
+      <c r="E3">
+        <v>7.1800000000000003E-2</v>
+      </c>
+      <c r="F3">
+        <v>336.40620000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>0.77890000000000004</v>
+      </c>
+      <c r="D4">
+        <v>49.514699999999998</v>
+      </c>
+      <c r="E4">
+        <v>7.0900000000000005E-2</v>
+      </c>
+      <c r="F4">
+        <v>31.116199999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>0.87309999999999999</v>
+      </c>
+      <c r="D5">
+        <v>3.1781000000000001</v>
+      </c>
+      <c r="E5">
+        <v>0.154</v>
+      </c>
+      <c r="F5">
+        <v>2.1715</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>0.81540000000000001</v>
+      </c>
+      <c r="D6">
+        <v>660.88729999999998</v>
+      </c>
+      <c r="E6">
+        <v>0.15290000000000001</v>
+      </c>
+      <c r="F6">
+        <v>465.59859999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0.76449999999999996</v>
+      </c>
+      <c r="D7">
+        <v>171.05240000000001</v>
+      </c>
+      <c r="E7">
+        <v>0.68410000000000004</v>
+      </c>
+      <c r="F7">
+        <v>115.4483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove obsolete CSV and Excel files related to molecular comparisons. Update the main comparison CSV to reflect new data entries and improve accuracy in predicted properties. Enhance the MolecularOptimizationAgent with a new parameter for CLI logging of RAG actions, improving traceability during optimization processes. Update requirements to include additional libraries for unstructured document processing.
</commit_message>
<xml_diff>
--- a/prediction results.xlsx
+++ b/prediction results.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cursor Projects\EnergeticGraph\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07049A9-07FD-45BF-93C6-6ABD6146BDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0827AD4A-4CB0-47B2-9FCE-63459C847C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="6100" windowWidth="28800" windowHeight="15370" activeTab="4" xr2:uid="{89EC946F-DC53-429F-91F6-32650855A236}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{89EC946F-DC53-429F-91F6-32650855A236}"/>
   </bookViews>
   <sheets>
     <sheet name="Kernel Ridge" sheetId="1" r:id="rId1"/>
     <sheet name="SVR" sheetId="2" r:id="rId2"/>
     <sheet name="Random Forest" sheetId="3" r:id="rId3"/>
     <sheet name="XGBoost" sheetId="4" r:id="rId4"/>
-    <sheet name="XGBoost (Coulomb)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="12">
   <si>
     <t>property</t>
   </si>
@@ -1085,162 +1084,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689E851C-92EB-4238-AD5F-CA3B296E8810}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.90625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>0.98009999999999997</v>
-      </c>
-      <c r="C2">
-        <v>0.81299999999999994</v>
-      </c>
-      <c r="D2">
-        <v>6.2E-2</v>
-      </c>
-      <c r="E2">
-        <v>3.7699999999999997E-2</v>
-      </c>
-      <c r="F2">
-        <v>4.7600000000000003E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>0.89029999999999998</v>
-      </c>
-      <c r="D3">
-        <v>489.19229999999999</v>
-      </c>
-      <c r="E3">
-        <v>7.1800000000000003E-2</v>
-      </c>
-      <c r="F3">
-        <v>336.40620000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>0.77890000000000004</v>
-      </c>
-      <c r="D4">
-        <v>49.514699999999998</v>
-      </c>
-      <c r="E4">
-        <v>7.0900000000000005E-2</v>
-      </c>
-      <c r="F4">
-        <v>31.116199999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>0.87309999999999999</v>
-      </c>
-      <c r="D5">
-        <v>3.1781000000000001</v>
-      </c>
-      <c r="E5">
-        <v>0.154</v>
-      </c>
-      <c r="F5">
-        <v>2.1715</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>0.81540000000000001</v>
-      </c>
-      <c r="D6">
-        <v>660.88729999999998</v>
-      </c>
-      <c r="E6">
-        <v>0.15290000000000001</v>
-      </c>
-      <c r="F6">
-        <v>465.59859999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>0.76449999999999996</v>
-      </c>
-      <c r="D7">
-        <v>171.05240000000001</v>
-      </c>
-      <c r="E7">
-        <v>0.68410000000000004</v>
-      </c>
-      <c r="F7">
-        <v>115.4483</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>